<commit_message>
fix(core): keep checkbox renderers formula-friendly
</commit_message>
<xml_diff>
--- a/packages/examples/showcase/kitchen-sink/artifact/kitchen-sink.xlsx
+++ b/packages/examples/showcase/kitchen-sink/artifact/kitchen-sink.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="209">
   <si>
     <t>Kitchen Sink Feature Map</t>
   </si>
@@ -63,9 +63,6 @@
     <t>accessor, dot paths, callbacks, defaultValue, autoWidth</t>
   </si>
   <si>
-    <t>☑</t>
-  </si>
-  <si>
     <t>Sub-row expansion</t>
   </si>
   <si>
@@ -336,9 +333,6 @@
     <t>Premium support extension</t>
   </si>
   <si>
-    <t>☐</t>
-  </si>
-  <si>
     <t>ORD-1002</t>
   </si>
   <si>
@@ -492,7 +486,7 @@
     <t>Medium</t>
   </si>
   <si>
-    <t>N/A</t>
+    <t/>
   </si>
   <si>
     <t>At risk</t>
@@ -661,11 +655,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="166" formatCode="0%"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
+  <numFmts count="6">
+    <numFmt numFmtId="164" formatCode="&quot;☑&quot;;;&quot;☐&quot;;&quot;&quot;"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="0%"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="169" formatCode="&quot;☑&quot;;;&quot;☐&quot;;&quot;N/A&quot;"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -856,7 +852,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -876,7 +872,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -894,10 +890,10 @@
     <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -906,37 +902,40 @@
     <xf numFmtId="0" fontId="10" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="10" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="12" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="12" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -949,18 +948,18 @@
       <alignment vertical="center"/>
       <protection/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="12" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1211,11 +1210,11 @@
       <c r="E3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>13</v>
+      <c r="F3" s="7">
+        <v>1</v>
+      </c>
+      <c r="G3" s="7">
+        <v>1</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
@@ -1223,68 +1222,68 @@
         <v>8</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>13</v>
+      <c r="F4" s="7">
+        <v>1</v>
+      </c>
+      <c r="G4" s="7">
+        <v>1</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>13</v>
+      <c r="F5" s="7">
+        <v>1</v>
+      </c>
+      <c r="G5" s="7">
+        <v>1</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>13</v>
+      <c r="F6" s="7">
+        <v>1</v>
+      </c>
+      <c r="G6" s="7">
+        <v>1</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
@@ -1292,206 +1291,206 @@
         <v>8</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>13</v>
+      <c r="F7" s="7">
+        <v>1</v>
+      </c>
+      <c r="G7" s="7">
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="E8" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>13</v>
+      <c r="F8" s="7">
+        <v>1</v>
+      </c>
+      <c r="G8" s="7">
+        <v>1</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="E9" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>13</v>
+      <c r="F9" s="7">
+        <v>1</v>
+      </c>
+      <c r="G9" s="7">
+        <v>1</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="E10" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E10" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>13</v>
+      <c r="F10" s="7">
+        <v>1</v>
+      </c>
+      <c r="G10" s="7">
+        <v>1</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="E11" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>13</v>
+      <c r="F11" s="7">
+        <v>1</v>
+      </c>
+      <c r="G11" s="7">
+        <v>1</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="C12" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="D12" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="E12" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E12" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>13</v>
+      <c r="F12" s="7">
+        <v>1</v>
+      </c>
+      <c r="G12" s="7">
+        <v>1</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="E13" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="E13" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>13</v>
+      <c r="F13" s="7">
+        <v>1</v>
+      </c>
+      <c r="G13" s="7">
+        <v>1</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="E14" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="E14" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>13</v>
+      <c r="F14" s="7">
+        <v>1</v>
+      </c>
+      <c r="G14" s="7">
+        <v>1</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="E15" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="E15" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>13</v>
+      <c r="F15" s="7">
+        <v>1</v>
+      </c>
+      <c r="G15" s="7">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1533,7 +1532,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1545,28 +1544,28 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="F2" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>185</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1">
@@ -1575,19 +1574,19 @@
         <f>IMAGE("https://dummyimage.com/48x48/1e40af/ffffff.png&amp;text=BK","Atlas Field Backpack",3,44,44)</f>
       </c>
       <c r="C3" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>190</v>
-      </c>
       <c r="F3" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>13</v>
+        <v>151</v>
+      </c>
+      <c r="G3" s="7">
+        <v>1</v>
       </c>
       <c r="H3" s="13">
         <v>129</v>
@@ -1599,19 +1598,19 @@
         <f>IMAGE("https://dummyimage.com/48x48/065f46/ffffff.png&amp;text=EL","Pulse USB-C Dock",3,44,44)</f>
       </c>
       <c r="C4" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>193</v>
-      </c>
       <c r="F4" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>13</v>
+        <v>149</v>
+      </c>
+      <c r="G4" s="7">
+        <v>1</v>
       </c>
       <c r="H4" s="13">
         <v>189</v>
@@ -1623,19 +1622,19 @@
         <f>IMAGE("https://dummyimage.com/48x48/92400e/ffffff.png&amp;text=HM","Northstar Desk Lamp",3,44,44)</f>
       </c>
       <c r="C5" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="F5" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>197</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>104</v>
+      <c r="G5" s="7">
+        <v>0</v>
       </c>
       <c r="H5" s="13">
         <v>74</v>
@@ -1667,7 +1666,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1675,24 +1674,24 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C3" s="13">
         <v>42000</v>
@@ -1703,10 +1702,10 @@
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C4" s="13">
         <v>18000</v>
@@ -1717,10 +1716,10 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C5" s="13">
         <v>12000</v>
@@ -1731,7 +1730,7 @@
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="C6" s="16" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
@@ -1770,52 +1769,52 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="30" t="s">
-        <v>76</v>
-      </c>
-      <c r="B3" s="31">
+      <c r="A3" s="31" t="s">
+        <v>75</v>
+      </c>
+      <c r="B3" s="32">
         <v>42000</v>
       </c>
-      <c r="C3" s="32">
+      <c r="C3" s="33">
         <f>ROUND((B3*0.9),0)</f>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="30" t="s">
-        <v>81</v>
-      </c>
-      <c r="B4" s="31">
+      <c r="A4" s="31" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" s="32">
         <v>18000</v>
       </c>
-      <c r="C4" s="32">
+      <c r="C4" s="33">
         <f>ROUND((B4*0.9),0)</f>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="30" t="s">
-        <v>86</v>
-      </c>
-      <c r="B5" s="31">
+      <c r="A5" s="31" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" s="32">
         <v>12000</v>
       </c>
-      <c r="C5" s="32">
+      <c r="C5" s="33">
         <f>ROUND((B5*0.9),0)</f>
       </c>
     </row>
@@ -1848,30 +1847,30 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="23" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B1" s="23" t="s">
+        <v>122</v>
+      </c>
+      <c r="C1" s="23" t="s">
+        <v>205</v>
+      </c>
+      <c r="D1" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="E1" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="C1" s="23" t="s">
-        <v>207</v>
-      </c>
-      <c r="D1" s="23" t="s">
+      <c r="F1" s="23" t="s">
         <v>125</v>
-      </c>
-      <c r="E1" s="23" t="s">
-        <v>126</v>
-      </c>
-      <c r="F1" s="23" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C2" s="15">
         <v>8</v>
@@ -1889,10 +1888,10 @@
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C3" s="15">
         <v>24</v>
@@ -1910,10 +1909,10 @@
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C4" s="15">
         <v>14</v>
@@ -1931,9 +1930,9 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="25" t="s">
-        <v>112</v>
-      </c>
-      <c r="C5" s="33">
+        <v>110</v>
+      </c>
+      <c r="C5" s="34">
         <f>SUBTOTAL(109,[Units])</f>
         <v>46</v>
       </c>
@@ -1945,8 +1944,8 @@
         <f>SUBTOTAL(109,[Cost])</f>
         <v>15280</v>
       </c>
-      <c r="F5" s="34" t="s">
-        <v>208</v>
+      <c r="F5" s="35" t="s">
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -1974,13 +1973,13 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="G1" s="1" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
@@ -1989,39 +1988,39 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="I2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C3" s="13">
         <v>420000</v>
@@ -2030,13 +2029,13 @@
         <v>46042.395833333336</v>
       </c>
       <c r="G3" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="H3" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>76</v>
-      </c>
       <c r="I3" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J3" s="13">
         <v>420000</v>
@@ -2047,10 +2046,10 @@
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C4" s="13">
         <v>96000</v>
@@ -2059,13 +2058,13 @@
         <v>46046.395833333336</v>
       </c>
       <c r="G4" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>81</v>
-      </c>
       <c r="I4" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J4" s="13">
         <v>96000</v>
@@ -2076,10 +2075,10 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C5" s="13">
         <v>18000</v>
@@ -2088,13 +2087,13 @@
         <v>46050.395833333336</v>
       </c>
       <c r="G5" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H5" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="H5" s="4" t="s">
-        <v>86</v>
-      </c>
       <c r="I5" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J5" s="13">
         <v>18000</v>
@@ -2127,7 +2126,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2138,39 +2137,39 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>78</v>
       </c>
       <c r="E3" s="13">
         <v>420000</v>
@@ -2179,21 +2178,21 @@
         <v>46042.395833333336</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="8" t="s">
         <v>82</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>83</v>
       </c>
       <c r="E4" s="13">
         <v>96000</v>
@@ -2202,21 +2201,21 @@
         <v>46046.395833333336</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="11" t="s">
         <v>87</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>88</v>
       </c>
       <c r="E5" s="13">
         <v>18000</v>
@@ -2225,7 +2224,7 @@
         <v>46050.395833333336</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -2253,7 +2252,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2266,48 +2265,48 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="6" t="s">
         <v>100</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>101</v>
       </c>
       <c r="F3" s="15">
         <v>8</v>
@@ -2318,8 +2317,8 @@
       <c r="H3" s="13">
         <v>11600</v>
       </c>
-      <c r="I3" s="7" t="s">
-        <v>13</v>
+      <c r="I3" s="7">
+        <v>1</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
@@ -2327,10 +2326,10 @@
       <c r="B4" s="4"/>
       <c r="C4" s="3"/>
       <c r="D4" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>102</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>103</v>
       </c>
       <c r="F4" s="15">
         <v>1</v>
@@ -2341,25 +2340,25 @@
       <c r="H4" s="13">
         <v>950</v>
       </c>
-      <c r="I4" s="7" t="s">
-        <v>104</v>
+      <c r="I4" s="7">
+        <v>0</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>105</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>107</v>
       </c>
       <c r="F5" s="15">
         <v>24</v>
@@ -2370,8 +2369,8 @@
       <c r="H5" s="13">
         <v>1896</v>
       </c>
-      <c r="I5" s="7" t="s">
-        <v>13</v>
+      <c r="I5" s="7">
+        <v>1</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
@@ -2379,10 +2378,10 @@
       <c r="B6" s="4"/>
       <c r="C6" s="8"/>
       <c r="D6" s="4" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F6" s="15">
         <v>2</v>
@@ -2393,8 +2392,8 @@
       <c r="H6" s="13">
         <v>2500</v>
       </c>
-      <c r="I6" s="7" t="s">
-        <v>13</v>
+      <c r="I6" s="7">
+        <v>1</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
@@ -2402,10 +2401,10 @@
       <c r="B7" s="4"/>
       <c r="C7" s="8"/>
       <c r="D7" s="4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F7" s="15">
         <v>1</v>
@@ -2416,13 +2415,13 @@
       <c r="H7" s="13">
         <v>600</v>
       </c>
-      <c r="I7" s="7" t="s">
-        <v>104</v>
+      <c r="I7" s="7">
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="16" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F8" s="16">
         <v>36</v>
@@ -2463,7 +2462,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2477,39 +2476,39 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B3" s="15">
         <v>8</v>
@@ -2541,7 +2540,7 @@
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B4" s="15">
         <v>24</v>
@@ -2573,7 +2572,7 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B5" s="15">
         <v>14</v>
@@ -2642,7 +2641,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2653,33 +2652,33 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C3" s="13">
         <v>420000</v>
@@ -2699,10 +2698,10 @@
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C4" s="13">
         <v>96000</v>
@@ -2722,10 +2721,10 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C5" s="13">
         <v>18000</v>
@@ -2745,10 +2744,10 @@
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C6" s="13">
         <v>260000</v>
@@ -2768,7 +2767,7 @@
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="16" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B7" s="16"/>
       <c r="C7" s="17">
@@ -2787,10 +2786,10 @@
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="16" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C8" s="17">
         <f>AVERAGE(C3:C6)</f>
@@ -2832,39 +2831,39 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="23" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="23" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="D1" s="23" t="s">
+        <v>129</v>
+      </c>
+      <c r="E1" s="23" t="s">
+        <v>128</v>
+      </c>
+      <c r="F1" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="G1" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="H1" s="23" t="s">
         <v>138</v>
-      </c>
-      <c r="D1" s="23" t="s">
-        <v>131</v>
-      </c>
-      <c r="E1" s="23" t="s">
-        <v>130</v>
-      </c>
-      <c r="F1" s="23" t="s">
-        <v>132</v>
-      </c>
-      <c r="G1" s="23" t="s">
-        <v>139</v>
-      </c>
-      <c r="H1" s="23" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>141</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>143</v>
       </c>
       <c r="D2" s="13">
         <v>320000</v>
@@ -2886,13 +2885,13 @@
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D3" s="13">
         <v>42000</v>
@@ -2914,13 +2913,13 @@
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D4" s="13">
         <v>18000</v>
@@ -2942,7 +2941,7 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="25" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D5" s="26">
         <f>SUBTOTAL(109,[AMER])</f>
@@ -2986,7 +2985,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2995,70 +2994,70 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>150</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>154</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>13</v>
+        <v>152</v>
+      </c>
+      <c r="D3" s="7">
+        <v>1</v>
+      </c>
+      <c r="E3" s="28">
+        <v>1</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>156</v>
+        <v>153</v>
+      </c>
+      <c r="D4" s="7">
+        <v>0</v>
+      </c>
+      <c r="E4" s="28" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="B5" s="28" t="s">
-        <v>157</v>
+        <v>131</v>
+      </c>
+      <c r="B5" s="29" t="s">
+        <v>155</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>154</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>104</v>
+        <v>152</v>
+      </c>
+      <c r="D5" s="7">
+        <v>0</v>
+      </c>
+      <c r="E5" s="28">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3080,53 +3079,53 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>159</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -3172,7 +3171,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3191,80 +3190,80 @@
       <c r="P1" s="1"/>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="29"/>
+      <c r="A2" s="30"/>
       <c r="B2" s="23" t="s">
-        <v>169</v>
-      </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
+        <v>167</v>
+      </c>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
       <c r="J2" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="K2" s="29"/>
-      <c r="L2" s="29"/>
-      <c r="M2" s="29"/>
-      <c r="N2" s="29"/>
-      <c r="O2" s="29"/>
-      <c r="P2" s="29"/>
+        <v>168</v>
+      </c>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30"/>
+      <c r="N2" s="30"/>
+      <c r="O2" s="30"/>
+      <c r="P2" s="30"/>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="J3" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="P3" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="P3" s="2" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B4" s="4">
         <v>82</v>
@@ -3308,7 +3307,7 @@
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B5" s="4">
         <v>44</v>
@@ -3352,7 +3351,7 @@
     </row>
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B6" s="4">
         <v>68</v>

</xml_diff>

<commit_message>
test(examples): showcase checkbox-driven workbook logic
</commit_message>
<xml_diff>
--- a/packages/examples/showcase/kitchen-sink/artifact/kitchen-sink.xlsx
+++ b/packages/examples/showcase/kitchen-sink/artifact/kitchen-sink.xlsx
@@ -123,10 +123,10 @@
     <t>06 Badges Checkboxes</t>
   </si>
   <si>
-    <t>Status labels and boolean checks are ordinary styled cells.</t>
-  </si>
-  <si>
-    <t>type: badge, type: checkbox</t>
+    <t>Checkbox toggles feed live formulas and conditional styles; locked checkbox cells stay disabled on the protected sheet.</t>
+  </si>
+  <si>
+    <t>type: badge, type: checkbox, refs.column(), conditionalStyle, protection.locked</t>
   </si>
   <si>
     <t>Hyperlinks</t>
@@ -462,9 +462,6 @@
     <t>Hana Sato</t>
   </si>
   <si>
-    <t>Badge and Checkbox Renderers</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
@@ -477,16 +474,19 @@
     <t>Billing</t>
   </si>
   <si>
+    <t>Live Decision</t>
+  </si>
+  <si>
     <t>Live</t>
   </si>
   <si>
     <t>High</t>
   </si>
   <si>
+    <t>Launching</t>
+  </si>
+  <si>
     <t>Medium</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>At risk</t>
@@ -655,15 +655,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
-    <numFmt numFmtId="164" formatCode="&quot;☑&quot;;;&quot;☐&quot;;&quot;&quot;"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="167" formatCode="0%"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
-    <numFmt numFmtId="169" formatCode="&quot;☑&quot;;;&quot;☐&quot;;&quot;N/A&quot;"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="166" formatCode="0%"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -721,10 +719,18 @@
     </font>
     <font>
       <b/>
+      <color rgb="FF475569"/>
+    </font>
+    <font>
+      <b/>
       <color rgb="FF991B1B"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FF64748B"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -799,6 +805,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFEE2E2"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -852,7 +864,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -872,8 +884,13 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -890,10 +907,10 @@
     <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -902,71 +919,98 @@
     <xf numFmtId="0" fontId="10" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="10" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="10" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="10" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <protection/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="12" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="5">
     <dxf>
       <font>
         <b/>
@@ -997,6 +1041,28 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFEDD5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF92400E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF475569"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF1F5F9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1108,6 +1174,23 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DynamicTerritoryMatrix" displayName="DynamicTerritoryMatrix" ref="A1:H5" totalsRowCount="1" headerRowCount="1">
   <autoFilter ref="A1:H4"/>
@@ -1154,8 +1237,8 @@
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="27" customWidth="1"/>
     <col min="3" max="3" width="29" customWidth="1"/>
-    <col min="4" max="4" width="75" customWidth="1"/>
-    <col min="5" max="5" width="69" customWidth="1"/>
+    <col min="4" max="4" width="124" customWidth="1"/>
+    <col min="5" max="5" width="84" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
   </cols>
@@ -1210,10 +1293,10 @@
       <c r="E3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G3" s="7">
+      <c r="G3" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1233,10 +1316,10 @@
       <c r="E4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1256,10 +1339,10 @@
       <c r="E5" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1279,10 +1362,10 @@
       <c r="E6" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1302,10 +1385,10 @@
       <c r="E7" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1325,10 +1408,10 @@
       <c r="E8" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1348,10 +1431,10 @@
       <c r="E9" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1371,10 +1454,10 @@
       <c r="E10" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1394,10 +1477,10 @@
       <c r="E11" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="F11" s="7">
+      <c r="F11" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1417,10 +1500,10 @@
       <c r="E12" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="F12" s="7">
+      <c r="F12" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G12" s="7">
+      <c r="G12" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1440,10 +1523,10 @@
       <c r="E13" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="F13" s="7">
+      <c r="F13" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G13" s="7">
+      <c r="G13" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1463,10 +1546,10 @@
       <c r="E14" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="F14" s="7">
+      <c r="F14" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G14" s="7">
+      <c r="G14" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1486,10 +1569,10 @@
       <c r="E15" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="F15" s="7">
+      <c r="F15" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G15" s="7">
+      <c r="G15" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1559,7 +1642,7 @@
         <v>183</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>184</v>
@@ -1585,7 +1668,7 @@
       <c r="F3" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="G3" s="7">
+      <c r="G3" s="7" t="b">
         <v>1</v>
       </c>
       <c r="H3" s="13">
@@ -1607,9 +1690,9 @@
         <v>191</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="G4" s="7">
+        <v>148</v>
+      </c>
+      <c r="G4" s="7" t="b">
         <v>1</v>
       </c>
       <c r="H4" s="13">
@@ -1633,7 +1716,7 @@
       <c r="F5" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="7" t="b">
         <v>0</v>
       </c>
       <c r="H5" s="13">
@@ -1677,7 +1760,7 @@
         <v>68</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>197</v>
@@ -1786,35 +1869,35 @@
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="34" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="32">
+      <c r="B3" s="35">
         <v>42000</v>
       </c>
-      <c r="C3" s="33">
+      <c r="C3" s="36">
         <f>ROUND((B3*0.9),0)</f>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="31" t="s">
+      <c r="A4" s="34" t="s">
         <v>80</v>
       </c>
-      <c r="B4" s="32">
+      <c r="B4" s="35">
         <v>18000</v>
       </c>
-      <c r="C4" s="33">
+      <c r="C4" s="36">
         <f>ROUND((B4*0.9),0)</f>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="34" t="s">
         <v>85</v>
       </c>
-      <c r="B5" s="32">
+      <c r="B5" s="35">
         <v>12000</v>
       </c>
-      <c r="C5" s="33">
+      <c r="C5" s="36">
         <f>ROUND((B5*0.9),0)</f>
       </c>
     </row>
@@ -1932,7 +2015,7 @@
       <c r="A5" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="C5" s="34">
+      <c r="C5" s="37">
         <f>SUBTOTAL(109,[Units])</f>
         <v>46</v>
       </c>
@@ -1944,7 +2027,7 @@
         <f>SUBTOTAL(109,[Cost])</f>
         <v>15280</v>
       </c>
-      <c r="F5" s="35" t="s">
+      <c r="F5" s="38" t="s">
         <v>206</v>
       </c>
     </row>
@@ -2317,7 +2400,7 @@
       <c r="H3" s="13">
         <v>11600</v>
       </c>
-      <c r="I3" s="7">
+      <c r="I3" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2340,7 +2423,7 @@
       <c r="H4" s="13">
         <v>950</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="7" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2369,7 +2452,7 @@
       <c r="H5" s="13">
         <v>1896</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2392,7 +2475,7 @@
       <c r="H6" s="13">
         <v>2500</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2415,7 +2498,7 @@
       <c r="H7" s="13">
         <v>600</v>
       </c>
-      <c r="I7" s="7">
+      <c r="I7" s="7" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2973,7 +3056,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
@@ -2981,89 +3064,100 @@
     <col min="3" max="3" width="17" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="23" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="C1" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>150</v>
+      </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>150</v>
+      <c r="A2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="C2" s="27" t="s">
+        <v>152</v>
+      </c>
+      <c r="D2" s="28" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" s="29" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" s="30">
+        <f>IF(AND((D2=TRUE),(E2=TRUE)),"Ready",IF((D2=TRUE),"Billing hold","Waiting"))</f>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="C3" s="27" t="s">
-        <v>152</v>
-      </c>
-      <c r="D3" s="7">
-        <v>1</v>
-      </c>
-      <c r="E3" s="28">
-        <v>1</v>
+        <v>79</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="D3" s="28" t="b">
+        <v>0</v>
+      </c>
+      <c r="E3" s="29"/>
+      <c r="F3" s="30">
+        <f>IF(AND((D3=TRUE),(E3=TRUE)),"Ready",IF((D3=TRUE),"Billing hold","Waiting"))</f>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="D4" s="7">
+        <v>131</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>152</v>
+      </c>
+      <c r="D4" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="28" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="B5" s="29" t="s">
-        <v>155</v>
-      </c>
-      <c r="C5" s="27" t="s">
-        <v>152</v>
-      </c>
-      <c r="D5" s="7">
+      <c r="E4" s="29" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="28">
-        <v>0</v>
+      <c r="F4" s="30">
+        <f>IF(AND((D4=TRUE),(E4=TRUE)),"Ready",IF((D4=TRUE),"Billing hold","Waiting"))</f>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
+  <sheetProtection sheet="1" password="C6EC" selectLockedCells="1"/>
+  <conditionalFormatting sqref="F2:F4">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>AND((D2=TRUE),(E2=TRUE))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="2">
+      <formula>AND((D2=TRUE),(E2&lt;&gt;TRUE))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="3">
+      <formula>(D2&lt;&gt;TRUE)</formula>
+    </cfRule>
+  </conditionalFormatting>
 </worksheet>
 </file>
 
@@ -3190,26 +3284,26 @@
       <c r="P1" s="1"/>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="30"/>
+      <c r="A2" s="33"/>
       <c r="B2" s="23" t="s">
         <v>167</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
       <c r="J2" s="23" t="s">
         <v>168</v>
       </c>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="30"/>
-      <c r="O2" s="30"/>
-      <c r="P2" s="30"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="33"/>
+      <c r="M2" s="33"/>
+      <c r="N2" s="33"/>
+      <c r="O2" s="33"/>
+      <c r="P2" s="33"/>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="s">

</xml_diff>